<commit_message>
Complete data mapping quality checks project
</commit_message>
<xml_diff>
--- a/input/sample_data_mapping_workbook.xlsx
+++ b/input/sample_data_mapping_workbook.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30224"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E90F784A-287D-468E-8D64-9116795B6322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9172B864-6736-4F5C-B5E6-C7E8FB1953B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="14" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>

</xml_diff>